<commit_message>
Agregar indicador SPI/PIB anual en Área de Intervención 1
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/areas_intervencion.xlsx
+++ b/data/areas_intervencion.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\crdavila\Inclusión Financiera\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4BA9B21-2E25-40D7-ABEF-A2062CA778DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F81209E-1126-4ACD-93E9-716CC644716A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{5E598A90-010E-43CD-AAA8-B76B1F3B89A4}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{5E598A90-010E-43CD-AAA8-B76B1F3B89A4}"/>
   </bookViews>
   <sheets>
     <sheet name="Intervención 1" sheetId="3" r:id="rId1"/>
-    <sheet name="Intervención 2" sheetId="4" r:id="rId2"/>
-    <sheet name="Intervención 3" sheetId="1" r:id="rId3"/>
-    <sheet name="Intervención 4" sheetId="6" r:id="rId4"/>
+    <sheet name="Intervención 1 - Anual" sheetId="7" r:id="rId2"/>
+    <sheet name="Intervención 2" sheetId="4" r:id="rId3"/>
+    <sheet name="Intervención 3" sheetId="1" r:id="rId4"/>
+    <sheet name="Intervención 4" sheetId="6" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="57">
   <si>
     <t>ÁREA DE INTERVENCIÓN 1: Puntos de acceso y canales</t>
   </si>
@@ -205,6 +206,12 @@
   <si>
     <t>Quejas y reclamos resueltos SB</t>
   </si>
+  <si>
+    <t>Año</t>
+  </si>
+  <si>
+    <t>SPI / PIB</t>
+  </si>
 </sst>
 </file>
 
@@ -277,7 +284,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -309,13 +316,39 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="0"/>
+      </left>
+      <right style="thin">
+        <color theme="0"/>
+      </right>
+      <top style="thin">
+        <color theme="0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0"/>
+      </left>
+      <right style="thin">
+        <color theme="0"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color theme="0"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -340,14 +373,23 @@
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -699,42 +741,42 @@
       </c>
     </row>
     <row r="2" spans="1:9">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="14" t="s">
+      <c r="B2" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
-      <c r="F2" s="14"/>
-      <c r="G2" s="14"/>
-      <c r="H2" s="14"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="15"/>
+      <c r="G2" s="15"/>
+      <c r="H2" s="15"/>
     </row>
     <row r="3" spans="1:9">
-      <c r="A3" s="16"/>
-      <c r="B3" s="15" t="s">
+      <c r="A3" s="14"/>
+      <c r="B3" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="14" t="s">
+      <c r="C3" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="14"/>
-      <c r="E3" s="14"/>
-      <c r="F3" s="15" t="s">
+      <c r="D3" s="15"/>
+      <c r="E3" s="15"/>
+      <c r="F3" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="G3" s="15" t="s">
+      <c r="G3" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="H3" s="15" t="s">
+      <c r="H3" s="16" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="22.5">
-      <c r="A4" s="16"/>
-      <c r="B4" s="15"/>
+      <c r="A4" s="14"/>
+      <c r="B4" s="16"/>
       <c r="C4" s="11" t="s">
         <v>8</v>
       </c>
@@ -744,9 +786,9 @@
       <c r="E4" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="F4" s="15"/>
-      <c r="G4" s="15"/>
-      <c r="H4" s="15"/>
+      <c r="F4" s="16"/>
+      <c r="G4" s="16"/>
+      <c r="H4" s="16"/>
     </row>
     <row r="5" spans="1:9">
       <c r="A5" s="7" t="s">
@@ -1515,6 +1557,152 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CB7830BF-E128-4321-BA84-2D470FBFAC90}">
+  <dimension ref="A1:B17"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="B1" s="17" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="16"/>
+      <c r="B2" s="18"/>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" s="19">
+        <v>2010</v>
+      </c>
+      <c r="B3" s="19">
+        <v>44.96</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" s="19">
+        <v>2011</v>
+      </c>
+      <c r="B4" s="19">
+        <v>49.85</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" s="19">
+        <v>2012</v>
+      </c>
+      <c r="B5" s="19">
+        <v>55.58</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" s="19">
+        <v>2013</v>
+      </c>
+      <c r="B6" s="19">
+        <v>60.65</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" s="19">
+        <v>2014</v>
+      </c>
+      <c r="B7" s="19">
+        <v>65.19</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" s="19">
+        <v>2015</v>
+      </c>
+      <c r="B8" s="19">
+        <v>89.82</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9" s="19">
+        <v>2016</v>
+      </c>
+      <c r="B9" s="19">
+        <v>93.82</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10" s="19">
+        <v>2017</v>
+      </c>
+      <c r="B10" s="19">
+        <v>94.73</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2">
+      <c r="A11" s="19">
+        <v>2018</v>
+      </c>
+      <c r="B11" s="19">
+        <v>100.27</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2">
+      <c r="A12" s="19">
+        <v>2019</v>
+      </c>
+      <c r="B12" s="19">
+        <v>105.45</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2">
+      <c r="A13" s="19">
+        <v>2020</v>
+      </c>
+      <c r="B13" s="19">
+        <v>115.37</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2">
+      <c r="A14" s="19">
+        <v>2021</v>
+      </c>
+      <c r="B14" s="19">
+        <v>127.74</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2">
+      <c r="A15" s="19">
+        <v>2022</v>
+      </c>
+      <c r="B15" s="19">
+        <v>134.66</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2">
+      <c r="A16" s="19">
+        <v>2023</v>
+      </c>
+      <c r="B16" s="19">
+        <v>136.80000000000001</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2">
+      <c r="A17" s="19">
+        <v>2024</v>
+      </c>
+      <c r="B17" s="19">
+        <v>139.55000000000001</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA07A8FE-F98F-4F5A-8C53-0373B7877FD2}">
   <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15"/>
@@ -1651,7 +1839,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC53E29E-3BCB-4B4F-89C6-6BE945E71D8E}">
   <sheetPr codeName="Hoja1"/>
   <dimension ref="A1:F160"/>
@@ -4832,7 +5020,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AC3F0BE7-B1BF-401F-81EA-ACF363BF306E}">
   <dimension ref="A1:B73"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15"/>

</xml_diff>

<commit_message>
Área 2: agregar sección Transferencias MDH con KPIs, gráficos por tipo, edad y evolución anual
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/areas_intervencion.xlsx
+++ b/data/areas_intervencion.xlsx
@@ -8,16 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\crdavila\Inclusión Financiera\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F81209E-1126-4ACD-93E9-716CC644716A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DAA3B31-9629-4083-8BA6-80A23A3B58C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{5E598A90-010E-43CD-AAA8-B76B1F3B89A4}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="3" xr2:uid="{5E598A90-010E-43CD-AAA8-B76B1F3B89A4}"/>
   </bookViews>
   <sheets>
     <sheet name="Intervención 1" sheetId="3" r:id="rId1"/>
     <sheet name="Intervención 1 - Anual" sheetId="7" r:id="rId2"/>
     <sheet name="Intervención 2" sheetId="4" r:id="rId3"/>
-    <sheet name="Intervención 3" sheetId="1" r:id="rId4"/>
-    <sheet name="Intervención 4" sheetId="6" r:id="rId5"/>
+    <sheet name="Intervención 2 - MDH" sheetId="8" r:id="rId4"/>
+    <sheet name="Intervención 3" sheetId="1" r:id="rId5"/>
+    <sheet name="Intervención 4" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="76">
   <si>
     <t>ÁREA DE INTERVENCIÓN 1: Puntos de acceso y canales</t>
   </si>
@@ -211,6 +212,63 @@
   </si>
   <si>
     <t>SPI / PIB</t>
+  </si>
+  <si>
+    <t>periodo</t>
+  </si>
+  <si>
+    <t>tipo_transferencia</t>
+  </si>
+  <si>
+    <t>edad</t>
+  </si>
+  <si>
+    <t>total</t>
+  </si>
+  <si>
+    <t>Bono de Desarrollo Humano</t>
+  </si>
+  <si>
+    <t>De 18-29</t>
+  </si>
+  <si>
+    <t>De 30-39</t>
+  </si>
+  <si>
+    <t>De 40-49</t>
+  </si>
+  <si>
+    <t>De 50-59</t>
+  </si>
+  <si>
+    <t>De 60-64</t>
+  </si>
+  <si>
+    <t>BDH con Componente Variable</t>
+  </si>
+  <si>
+    <t>Bono 1000 Días</t>
+  </si>
+  <si>
+    <t>Pensión Mis Mejores Años</t>
+  </si>
+  <si>
+    <t>De 65-74</t>
+  </si>
+  <si>
+    <t>De 75-84</t>
+  </si>
+  <si>
+    <t>De 85-99</t>
+  </si>
+  <si>
+    <t>Mayor o igual a 100</t>
+  </si>
+  <si>
+    <t>Pensión Toda una Vida</t>
+  </si>
+  <si>
+    <t>Bono Joaquín Gallegos Lara</t>
   </si>
 </sst>
 </file>
@@ -222,7 +280,7 @@
     <numFmt numFmtId="164" formatCode="_ * #,##0.0_ ;_ * \-#,##0.0_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="165" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -268,6 +326,14 @@
       <color theme="0"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -348,7 +414,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -373,6 +439,9 @@
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -388,9 +457,7 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Millares" xfId="1" builtinId="3"/>
@@ -741,42 +808,42 @@
       </c>
     </row>
     <row r="2" spans="1:9">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="15" t="s">
+      <c r="B2" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="15"/>
-      <c r="D2" s="15"/>
-      <c r="E2" s="15"/>
-      <c r="F2" s="15"/>
-      <c r="G2" s="15"/>
-      <c r="H2" s="15"/>
+      <c r="C2" s="16"/>
+      <c r="D2" s="16"/>
+      <c r="E2" s="16"/>
+      <c r="F2" s="16"/>
+      <c r="G2" s="16"/>
+      <c r="H2" s="16"/>
     </row>
     <row r="3" spans="1:9">
-      <c r="A3" s="14"/>
-      <c r="B3" s="16" t="s">
+      <c r="A3" s="15"/>
+      <c r="B3" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="15" t="s">
+      <c r="C3" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="15"/>
-      <c r="E3" s="15"/>
-      <c r="F3" s="16" t="s">
+      <c r="D3" s="16"/>
+      <c r="E3" s="16"/>
+      <c r="F3" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="G3" s="16" t="s">
+      <c r="G3" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="H3" s="16" t="s">
+      <c r="H3" s="17" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="22.5">
-      <c r="A4" s="14"/>
-      <c r="B4" s="16"/>
+      <c r="A4" s="15"/>
+      <c r="B4" s="17"/>
       <c r="C4" s="11" t="s">
         <v>8</v>
       </c>
@@ -786,9 +853,9 @@
       <c r="E4" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="F4" s="16"/>
-      <c r="G4" s="16"/>
-      <c r="H4" s="16"/>
+      <c r="F4" s="17"/>
+      <c r="G4" s="17"/>
+      <c r="H4" s="17"/>
     </row>
     <row r="5" spans="1:9">
       <c r="A5" s="7" t="s">
@@ -1562,134 +1629,134 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="17" t="s">
         <v>55</v>
       </c>
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="18" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="2" spans="1:2">
-      <c r="A2" s="16"/>
-      <c r="B2" s="18"/>
+      <c r="A2" s="17"/>
+      <c r="B2" s="19"/>
     </row>
     <row r="3" spans="1:2">
-      <c r="A3" s="19">
+      <c r="A3" s="14">
         <v>2010</v>
       </c>
-      <c r="B3" s="19">
+      <c r="B3" s="14">
         <v>44.96</v>
       </c>
     </row>
     <row r="4" spans="1:2">
-      <c r="A4" s="19">
+      <c r="A4" s="14">
         <v>2011</v>
       </c>
-      <c r="B4" s="19">
+      <c r="B4" s="14">
         <v>49.85</v>
       </c>
     </row>
     <row r="5" spans="1:2">
-      <c r="A5" s="19">
+      <c r="A5" s="14">
         <v>2012</v>
       </c>
-      <c r="B5" s="19">
+      <c r="B5" s="14">
         <v>55.58</v>
       </c>
     </row>
     <row r="6" spans="1:2">
-      <c r="A6" s="19">
+      <c r="A6" s="14">
         <v>2013</v>
       </c>
-      <c r="B6" s="19">
+      <c r="B6" s="14">
         <v>60.65</v>
       </c>
     </row>
     <row r="7" spans="1:2">
-      <c r="A7" s="19">
+      <c r="A7" s="14">
         <v>2014</v>
       </c>
-      <c r="B7" s="19">
+      <c r="B7" s="14">
         <v>65.19</v>
       </c>
     </row>
     <row r="8" spans="1:2">
-      <c r="A8" s="19">
+      <c r="A8" s="14">
         <v>2015</v>
       </c>
-      <c r="B8" s="19">
+      <c r="B8" s="14">
         <v>89.82</v>
       </c>
     </row>
     <row r="9" spans="1:2">
-      <c r="A9" s="19">
+      <c r="A9" s="14">
         <v>2016</v>
       </c>
-      <c r="B9" s="19">
+      <c r="B9" s="14">
         <v>93.82</v>
       </c>
     </row>
     <row r="10" spans="1:2">
-      <c r="A10" s="19">
+      <c r="A10" s="14">
         <v>2017</v>
       </c>
-      <c r="B10" s="19">
+      <c r="B10" s="14">
         <v>94.73</v>
       </c>
     </row>
     <row r="11" spans="1:2">
-      <c r="A11" s="19">
+      <c r="A11" s="14">
         <v>2018</v>
       </c>
-      <c r="B11" s="19">
+      <c r="B11" s="14">
         <v>100.27</v>
       </c>
     </row>
     <row r="12" spans="1:2">
-      <c r="A12" s="19">
+      <c r="A12" s="14">
         <v>2019</v>
       </c>
-      <c r="B12" s="19">
+      <c r="B12" s="14">
         <v>105.45</v>
       </c>
     </row>
     <row r="13" spans="1:2">
-      <c r="A13" s="19">
+      <c r="A13" s="14">
         <v>2020</v>
       </c>
-      <c r="B13" s="19">
+      <c r="B13" s="14">
         <v>115.37</v>
       </c>
     </row>
     <row r="14" spans="1:2">
-      <c r="A14" s="19">
+      <c r="A14" s="14">
         <v>2021</v>
       </c>
-      <c r="B14" s="19">
+      <c r="B14" s="14">
         <v>127.74</v>
       </c>
     </row>
     <row r="15" spans="1:2">
-      <c r="A15" s="19">
+      <c r="A15" s="14">
         <v>2022</v>
       </c>
-      <c r="B15" s="19">
+      <c r="B15" s="14">
         <v>134.66</v>
       </c>
     </row>
     <row r="16" spans="1:2">
-      <c r="A16" s="19">
+      <c r="A16" s="14">
         <v>2023</v>
       </c>
-      <c r="B16" s="19">
+      <c r="B16" s="14">
         <v>136.80000000000001</v>
       </c>
     </row>
     <row r="17" spans="1:2">
-      <c r="A17" s="19">
+      <c r="A17" s="14">
         <v>2024</v>
       </c>
-      <c r="B17" s="19">
+      <c r="B17" s="14">
         <v>139.55000000000001</v>
       </c>
     </row>
@@ -1840,6 +1907,1332 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCF0D2D6-B265-42DF-B352-4D448DFAA1B5}">
+  <dimension ref="A1:D94"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" s="20" t="s">
+        <v>57</v>
+      </c>
+      <c r="B1" s="20" t="s">
+        <v>58</v>
+      </c>
+      <c r="C1" s="20" t="s">
+        <v>59</v>
+      </c>
+      <c r="D1" s="20" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2">
+        <v>2023</v>
+      </c>
+      <c r="B2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C2" t="s">
+        <v>62</v>
+      </c>
+      <c r="D2">
+        <v>35629</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3">
+        <v>2023</v>
+      </c>
+      <c r="B3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C3" t="s">
+        <v>63</v>
+      </c>
+      <c r="D3">
+        <v>56958</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4">
+        <v>2023</v>
+      </c>
+      <c r="B4" t="s">
+        <v>61</v>
+      </c>
+      <c r="C4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D4">
+        <v>50631</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5">
+        <v>2023</v>
+      </c>
+      <c r="B5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C5" t="s">
+        <v>65</v>
+      </c>
+      <c r="D5">
+        <v>37725</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6">
+        <v>2023</v>
+      </c>
+      <c r="B6" t="s">
+        <v>61</v>
+      </c>
+      <c r="C6" t="s">
+        <v>66</v>
+      </c>
+      <c r="D6">
+        <v>17368</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7">
+        <v>2023</v>
+      </c>
+      <c r="B7" t="s">
+        <v>67</v>
+      </c>
+      <c r="C7" t="s">
+        <v>62</v>
+      </c>
+      <c r="D7">
+        <v>25890</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="A8">
+        <v>2023</v>
+      </c>
+      <c r="B8" t="s">
+        <v>67</v>
+      </c>
+      <c r="C8" t="s">
+        <v>63</v>
+      </c>
+      <c r="D8">
+        <v>44349</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
+      <c r="A9">
+        <v>2023</v>
+      </c>
+      <c r="B9" t="s">
+        <v>67</v>
+      </c>
+      <c r="C9" t="s">
+        <v>64</v>
+      </c>
+      <c r="D9">
+        <v>29764</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="A10">
+        <v>2023</v>
+      </c>
+      <c r="B10" t="s">
+        <v>67</v>
+      </c>
+      <c r="C10" t="s">
+        <v>65</v>
+      </c>
+      <c r="D10">
+        <v>10710</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
+      <c r="A11">
+        <v>2023</v>
+      </c>
+      <c r="B11" t="s">
+        <v>67</v>
+      </c>
+      <c r="C11" t="s">
+        <v>66</v>
+      </c>
+      <c r="D11">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4">
+      <c r="A12">
+        <v>2023</v>
+      </c>
+      <c r="B12" t="s">
+        <v>68</v>
+      </c>
+      <c r="C12" t="s">
+        <v>62</v>
+      </c>
+      <c r="D12">
+        <v>5149</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4">
+      <c r="A13">
+        <v>2023</v>
+      </c>
+      <c r="B13" t="s">
+        <v>68</v>
+      </c>
+      <c r="C13" t="s">
+        <v>63</v>
+      </c>
+      <c r="D13">
+        <v>992</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
+      <c r="A14">
+        <v>2023</v>
+      </c>
+      <c r="B14" t="s">
+        <v>68</v>
+      </c>
+      <c r="C14" t="s">
+        <v>64</v>
+      </c>
+      <c r="D14">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4">
+      <c r="A15">
+        <v>2023</v>
+      </c>
+      <c r="B15" t="s">
+        <v>69</v>
+      </c>
+      <c r="C15" t="s">
+        <v>70</v>
+      </c>
+      <c r="D15">
+        <v>49559</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4">
+      <c r="A16">
+        <v>2023</v>
+      </c>
+      <c r="B16" t="s">
+        <v>69</v>
+      </c>
+      <c r="C16" t="s">
+        <v>71</v>
+      </c>
+      <c r="D16">
+        <v>36762</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4">
+      <c r="A17">
+        <v>2023</v>
+      </c>
+      <c r="B17" t="s">
+        <v>69</v>
+      </c>
+      <c r="C17" t="s">
+        <v>72</v>
+      </c>
+      <c r="D17">
+        <v>17346</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4">
+      <c r="A18">
+        <v>2023</v>
+      </c>
+      <c r="B18" t="s">
+        <v>69</v>
+      </c>
+      <c r="C18" t="s">
+        <v>73</v>
+      </c>
+      <c r="D18">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4">
+      <c r="A19">
+        <v>2023</v>
+      </c>
+      <c r="B19" t="s">
+        <v>74</v>
+      </c>
+      <c r="C19" t="s">
+        <v>62</v>
+      </c>
+      <c r="D19">
+        <v>6984</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4">
+      <c r="A20">
+        <v>2023</v>
+      </c>
+      <c r="B20" t="s">
+        <v>74</v>
+      </c>
+      <c r="C20" t="s">
+        <v>63</v>
+      </c>
+      <c r="D20">
+        <v>4538</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4">
+      <c r="A21">
+        <v>2023</v>
+      </c>
+      <c r="B21" t="s">
+        <v>74</v>
+      </c>
+      <c r="C21" t="s">
+        <v>64</v>
+      </c>
+      <c r="D21">
+        <v>4404</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4">
+      <c r="A22">
+        <v>2023</v>
+      </c>
+      <c r="B22" t="s">
+        <v>74</v>
+      </c>
+      <c r="C22" t="s">
+        <v>65</v>
+      </c>
+      <c r="D22">
+        <v>4480</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4">
+      <c r="A23">
+        <v>2023</v>
+      </c>
+      <c r="B23" t="s">
+        <v>74</v>
+      </c>
+      <c r="C23" t="s">
+        <v>66</v>
+      </c>
+      <c r="D23">
+        <v>2322</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4">
+      <c r="A24">
+        <v>2023</v>
+      </c>
+      <c r="B24" t="s">
+        <v>75</v>
+      </c>
+      <c r="C24" t="s">
+        <v>62</v>
+      </c>
+      <c r="D24">
+        <v>9438</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4">
+      <c r="A25">
+        <v>2023</v>
+      </c>
+      <c r="B25" t="s">
+        <v>75</v>
+      </c>
+      <c r="C25" t="s">
+        <v>63</v>
+      </c>
+      <c r="D25">
+        <v>6050</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4">
+      <c r="A26">
+        <v>2023</v>
+      </c>
+      <c r="B26" t="s">
+        <v>75</v>
+      </c>
+      <c r="C26" t="s">
+        <v>64</v>
+      </c>
+      <c r="D26">
+        <v>5144</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4">
+      <c r="A27">
+        <v>2023</v>
+      </c>
+      <c r="B27" t="s">
+        <v>75</v>
+      </c>
+      <c r="C27" t="s">
+        <v>65</v>
+      </c>
+      <c r="D27">
+        <v>4608</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4">
+      <c r="A28">
+        <v>2023</v>
+      </c>
+      <c r="B28" t="s">
+        <v>75</v>
+      </c>
+      <c r="C28" t="s">
+        <v>66</v>
+      </c>
+      <c r="D28">
+        <v>2184</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4">
+      <c r="A29">
+        <v>2023</v>
+      </c>
+      <c r="B29" t="s">
+        <v>75</v>
+      </c>
+      <c r="C29" t="s">
+        <v>70</v>
+      </c>
+      <c r="D29">
+        <v>3310</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4">
+      <c r="A30">
+        <v>2023</v>
+      </c>
+      <c r="B30" t="s">
+        <v>75</v>
+      </c>
+      <c r="C30" t="s">
+        <v>71</v>
+      </c>
+      <c r="D30">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4">
+      <c r="A31">
+        <v>2023</v>
+      </c>
+      <c r="B31" t="s">
+        <v>75</v>
+      </c>
+      <c r="C31" t="s">
+        <v>72</v>
+      </c>
+      <c r="D31">
+        <v>1152</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4">
+      <c r="A32">
+        <v>2023</v>
+      </c>
+      <c r="B32" t="s">
+        <v>75</v>
+      </c>
+      <c r="C32" t="s">
+        <v>73</v>
+      </c>
+      <c r="D32">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4">
+      <c r="A33">
+        <v>2024</v>
+      </c>
+      <c r="B33" t="s">
+        <v>61</v>
+      </c>
+      <c r="C33" t="s">
+        <v>62</v>
+      </c>
+      <c r="D33">
+        <v>69702</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4">
+      <c r="A34">
+        <v>2024</v>
+      </c>
+      <c r="B34" t="s">
+        <v>61</v>
+      </c>
+      <c r="C34" t="s">
+        <v>63</v>
+      </c>
+      <c r="D34">
+        <v>111175</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4">
+      <c r="A35">
+        <v>2024</v>
+      </c>
+      <c r="B35" t="s">
+        <v>61</v>
+      </c>
+      <c r="C35" t="s">
+        <v>64</v>
+      </c>
+      <c r="D35">
+        <v>105628</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4">
+      <c r="A36">
+        <v>2024</v>
+      </c>
+      <c r="B36" t="s">
+        <v>61</v>
+      </c>
+      <c r="C36" t="s">
+        <v>65</v>
+      </c>
+      <c r="D36">
+        <v>81774</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4">
+      <c r="A37">
+        <v>2024</v>
+      </c>
+      <c r="B37" t="s">
+        <v>61</v>
+      </c>
+      <c r="C37" t="s">
+        <v>66</v>
+      </c>
+      <c r="D37">
+        <v>37634</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4">
+      <c r="A38">
+        <v>2024</v>
+      </c>
+      <c r="B38" t="s">
+        <v>67</v>
+      </c>
+      <c r="C38" t="s">
+        <v>62</v>
+      </c>
+      <c r="D38">
+        <v>47928</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4">
+      <c r="A39">
+        <v>2024</v>
+      </c>
+      <c r="B39" t="s">
+        <v>67</v>
+      </c>
+      <c r="C39" t="s">
+        <v>63</v>
+      </c>
+      <c r="D39">
+        <v>72652</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4">
+      <c r="A40">
+        <v>2024</v>
+      </c>
+      <c r="B40" t="s">
+        <v>67</v>
+      </c>
+      <c r="C40" t="s">
+        <v>64</v>
+      </c>
+      <c r="D40">
+        <v>49239</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4">
+      <c r="A41">
+        <v>2024</v>
+      </c>
+      <c r="B41" t="s">
+        <v>67</v>
+      </c>
+      <c r="C41" t="s">
+        <v>65</v>
+      </c>
+      <c r="D41">
+        <v>16959</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4">
+      <c r="A42">
+        <v>2024</v>
+      </c>
+      <c r="B42" t="s">
+        <v>67</v>
+      </c>
+      <c r="C42" t="s">
+        <v>66</v>
+      </c>
+      <c r="D42">
+        <v>1302</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4">
+      <c r="A43">
+        <v>2024</v>
+      </c>
+      <c r="B43" t="s">
+        <v>68</v>
+      </c>
+      <c r="C43" t="s">
+        <v>62</v>
+      </c>
+      <c r="D43">
+        <v>6839</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4">
+      <c r="A44">
+        <v>2024</v>
+      </c>
+      <c r="B44" t="s">
+        <v>68</v>
+      </c>
+      <c r="C44" t="s">
+        <v>63</v>
+      </c>
+      <c r="D44">
+        <v>1121</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4">
+      <c r="A45">
+        <v>2024</v>
+      </c>
+      <c r="B45" t="s">
+        <v>68</v>
+      </c>
+      <c r="C45" t="s">
+        <v>64</v>
+      </c>
+      <c r="D45">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4">
+      <c r="A46">
+        <v>2024</v>
+      </c>
+      <c r="B46" t="s">
+        <v>69</v>
+      </c>
+      <c r="C46" t="s">
+        <v>70</v>
+      </c>
+      <c r="D46">
+        <v>123216</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4">
+      <c r="A47">
+        <v>2024</v>
+      </c>
+      <c r="B47" t="s">
+        <v>69</v>
+      </c>
+      <c r="C47" t="s">
+        <v>71</v>
+      </c>
+      <c r="D47">
+        <v>81991</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4">
+      <c r="A48">
+        <v>2024</v>
+      </c>
+      <c r="B48" t="s">
+        <v>69</v>
+      </c>
+      <c r="C48" t="s">
+        <v>72</v>
+      </c>
+      <c r="D48">
+        <v>37395</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4">
+      <c r="A49">
+        <v>2024</v>
+      </c>
+      <c r="B49" t="s">
+        <v>69</v>
+      </c>
+      <c r="C49" t="s">
+        <v>73</v>
+      </c>
+      <c r="D49">
+        <v>661</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4">
+      <c r="A50">
+        <v>2024</v>
+      </c>
+      <c r="B50" t="s">
+        <v>74</v>
+      </c>
+      <c r="C50" t="s">
+        <v>62</v>
+      </c>
+      <c r="D50">
+        <v>15297</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4">
+      <c r="A51">
+        <v>2024</v>
+      </c>
+      <c r="B51" t="s">
+        <v>74</v>
+      </c>
+      <c r="C51" t="s">
+        <v>63</v>
+      </c>
+      <c r="D51">
+        <v>9584</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4">
+      <c r="A52">
+        <v>2024</v>
+      </c>
+      <c r="B52" t="s">
+        <v>74</v>
+      </c>
+      <c r="C52" t="s">
+        <v>64</v>
+      </c>
+      <c r="D52">
+        <v>9032</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4">
+      <c r="A53">
+        <v>2024</v>
+      </c>
+      <c r="B53" t="s">
+        <v>74</v>
+      </c>
+      <c r="C53" t="s">
+        <v>65</v>
+      </c>
+      <c r="D53">
+        <v>9334</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4">
+      <c r="A54">
+        <v>2024</v>
+      </c>
+      <c r="B54" t="s">
+        <v>74</v>
+      </c>
+      <c r="C54" t="s">
+        <v>66</v>
+      </c>
+      <c r="D54">
+        <v>4688</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4">
+      <c r="A55">
+        <v>2024</v>
+      </c>
+      <c r="B55" t="s">
+        <v>75</v>
+      </c>
+      <c r="C55" t="s">
+        <v>62</v>
+      </c>
+      <c r="D55">
+        <v>9776</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4">
+      <c r="A56">
+        <v>2024</v>
+      </c>
+      <c r="B56" t="s">
+        <v>75</v>
+      </c>
+      <c r="C56" t="s">
+        <v>63</v>
+      </c>
+      <c r="D56">
+        <v>6401</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4">
+      <c r="A57">
+        <v>2024</v>
+      </c>
+      <c r="B57" t="s">
+        <v>75</v>
+      </c>
+      <c r="C57" t="s">
+        <v>64</v>
+      </c>
+      <c r="D57">
+        <v>5472</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4">
+      <c r="A58">
+        <v>2024</v>
+      </c>
+      <c r="B58" t="s">
+        <v>75</v>
+      </c>
+      <c r="C58" t="s">
+        <v>65</v>
+      </c>
+      <c r="D58">
+        <v>4861</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4">
+      <c r="A59">
+        <v>2024</v>
+      </c>
+      <c r="B59" t="s">
+        <v>75</v>
+      </c>
+      <c r="C59" t="s">
+        <v>66</v>
+      </c>
+      <c r="D59">
+        <v>2358</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4">
+      <c r="A60">
+        <v>2024</v>
+      </c>
+      <c r="B60" t="s">
+        <v>75</v>
+      </c>
+      <c r="C60" t="s">
+        <v>70</v>
+      </c>
+      <c r="D60">
+        <v>3522</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4">
+      <c r="A61">
+        <v>2024</v>
+      </c>
+      <c r="B61" t="s">
+        <v>75</v>
+      </c>
+      <c r="C61" t="s">
+        <v>71</v>
+      </c>
+      <c r="D61">
+        <v>2083</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4">
+      <c r="A62">
+        <v>2024</v>
+      </c>
+      <c r="B62" t="s">
+        <v>75</v>
+      </c>
+      <c r="C62" t="s">
+        <v>72</v>
+      </c>
+      <c r="D62">
+        <v>1135</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4">
+      <c r="A63">
+        <v>2024</v>
+      </c>
+      <c r="B63" t="s">
+        <v>75</v>
+      </c>
+      <c r="C63" t="s">
+        <v>73</v>
+      </c>
+      <c r="D63">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4">
+      <c r="A64">
+        <v>2025</v>
+      </c>
+      <c r="B64" t="s">
+        <v>61</v>
+      </c>
+      <c r="C64" t="s">
+        <v>62</v>
+      </c>
+      <c r="D64">
+        <v>68975</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4">
+      <c r="A65">
+        <v>2025</v>
+      </c>
+      <c r="B65" t="s">
+        <v>61</v>
+      </c>
+      <c r="C65" t="s">
+        <v>63</v>
+      </c>
+      <c r="D65">
+        <v>120356</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4">
+      <c r="A66">
+        <v>2025</v>
+      </c>
+      <c r="B66" t="s">
+        <v>61</v>
+      </c>
+      <c r="C66" t="s">
+        <v>64</v>
+      </c>
+      <c r="D66">
+        <v>122173</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4">
+      <c r="A67">
+        <v>2025</v>
+      </c>
+      <c r="B67" t="s">
+        <v>61</v>
+      </c>
+      <c r="C67" t="s">
+        <v>65</v>
+      </c>
+      <c r="D67">
+        <v>92677</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4">
+      <c r="A68">
+        <v>2025</v>
+      </c>
+      <c r="B68" t="s">
+        <v>61</v>
+      </c>
+      <c r="C68" t="s">
+        <v>66</v>
+      </c>
+      <c r="D68">
+        <v>42250</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4">
+      <c r="A69">
+        <v>2025</v>
+      </c>
+      <c r="B69" t="s">
+        <v>67</v>
+      </c>
+      <c r="C69" t="s">
+        <v>62</v>
+      </c>
+      <c r="D69">
+        <v>57911</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4">
+      <c r="A70">
+        <v>2025</v>
+      </c>
+      <c r="B70" t="s">
+        <v>67</v>
+      </c>
+      <c r="C70" t="s">
+        <v>63</v>
+      </c>
+      <c r="D70">
+        <v>79903</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4">
+      <c r="A71">
+        <v>2025</v>
+      </c>
+      <c r="B71" t="s">
+        <v>67</v>
+      </c>
+      <c r="C71" t="s">
+        <v>64</v>
+      </c>
+      <c r="D71">
+        <v>53737</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4">
+      <c r="A72">
+        <v>2025</v>
+      </c>
+      <c r="B72" t="s">
+        <v>67</v>
+      </c>
+      <c r="C72" t="s">
+        <v>65</v>
+      </c>
+      <c r="D72">
+        <v>17406</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4">
+      <c r="A73">
+        <v>2025</v>
+      </c>
+      <c r="B73" t="s">
+        <v>67</v>
+      </c>
+      <c r="C73" t="s">
+        <v>66</v>
+      </c>
+      <c r="D73">
+        <v>1310</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4">
+      <c r="A74">
+        <v>2025</v>
+      </c>
+      <c r="B74" t="s">
+        <v>68</v>
+      </c>
+      <c r="C74" t="s">
+        <v>62</v>
+      </c>
+      <c r="D74">
+        <v>7153</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4">
+      <c r="A75">
+        <v>2025</v>
+      </c>
+      <c r="B75" t="s">
+        <v>68</v>
+      </c>
+      <c r="C75" t="s">
+        <v>63</v>
+      </c>
+      <c r="D75">
+        <v>1399</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4">
+      <c r="A76">
+        <v>2025</v>
+      </c>
+      <c r="B76" t="s">
+        <v>68</v>
+      </c>
+      <c r="C76" t="s">
+        <v>64</v>
+      </c>
+      <c r="D76">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4">
+      <c r="A77">
+        <v>2025</v>
+      </c>
+      <c r="B77" t="s">
+        <v>69</v>
+      </c>
+      <c r="C77" t="s">
+        <v>70</v>
+      </c>
+      <c r="D77">
+        <v>136949</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4">
+      <c r="A78">
+        <v>2025</v>
+      </c>
+      <c r="B78" t="s">
+        <v>69</v>
+      </c>
+      <c r="C78" t="s">
+        <v>71</v>
+      </c>
+      <c r="D78">
+        <v>92310</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4">
+      <c r="A79">
+        <v>2025</v>
+      </c>
+      <c r="B79" t="s">
+        <v>69</v>
+      </c>
+      <c r="C79" t="s">
+        <v>72</v>
+      </c>
+      <c r="D79">
+        <v>43595</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4">
+      <c r="A80">
+        <v>2025</v>
+      </c>
+      <c r="B80" t="s">
+        <v>69</v>
+      </c>
+      <c r="C80" t="s">
+        <v>73</v>
+      </c>
+      <c r="D80">
+        <v>872</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4">
+      <c r="A81">
+        <v>2025</v>
+      </c>
+      <c r="B81" t="s">
+        <v>74</v>
+      </c>
+      <c r="C81" t="s">
+        <v>62</v>
+      </c>
+      <c r="D81">
+        <v>17664</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4">
+      <c r="A82">
+        <v>2025</v>
+      </c>
+      <c r="B82" t="s">
+        <v>74</v>
+      </c>
+      <c r="C82" t="s">
+        <v>63</v>
+      </c>
+      <c r="D82">
+        <v>11112</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4">
+      <c r="A83">
+        <v>2025</v>
+      </c>
+      <c r="B83" t="s">
+        <v>74</v>
+      </c>
+      <c r="C83" t="s">
+        <v>64</v>
+      </c>
+      <c r="D83">
+        <v>10406</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4">
+      <c r="A84">
+        <v>2025</v>
+      </c>
+      <c r="B84" t="s">
+        <v>74</v>
+      </c>
+      <c r="C84" t="s">
+        <v>65</v>
+      </c>
+      <c r="D84">
+        <v>10371</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4">
+      <c r="A85">
+        <v>2025</v>
+      </c>
+      <c r="B85" t="s">
+        <v>74</v>
+      </c>
+      <c r="C85" t="s">
+        <v>66</v>
+      </c>
+      <c r="D85">
+        <v>5243</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4">
+      <c r="A86">
+        <v>2025</v>
+      </c>
+      <c r="B86" t="s">
+        <v>75</v>
+      </c>
+      <c r="C86" t="s">
+        <v>62</v>
+      </c>
+      <c r="D86">
+        <v>10222</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4">
+      <c r="A87">
+        <v>2025</v>
+      </c>
+      <c r="B87" t="s">
+        <v>75</v>
+      </c>
+      <c r="C87" t="s">
+        <v>63</v>
+      </c>
+      <c r="D87">
+        <v>6910</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4">
+      <c r="A88">
+        <v>2025</v>
+      </c>
+      <c r="B88" t="s">
+        <v>75</v>
+      </c>
+      <c r="C88" t="s">
+        <v>64</v>
+      </c>
+      <c r="D88">
+        <v>6129</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4">
+      <c r="A89">
+        <v>2025</v>
+      </c>
+      <c r="B89" t="s">
+        <v>75</v>
+      </c>
+      <c r="C89" t="s">
+        <v>65</v>
+      </c>
+      <c r="D89">
+        <v>5420</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4">
+      <c r="A90">
+        <v>2025</v>
+      </c>
+      <c r="B90" t="s">
+        <v>75</v>
+      </c>
+      <c r="C90" t="s">
+        <v>66</v>
+      </c>
+      <c r="D90">
+        <v>2687</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4">
+      <c r="A91">
+        <v>2025</v>
+      </c>
+      <c r="B91" t="s">
+        <v>75</v>
+      </c>
+      <c r="C91" t="s">
+        <v>70</v>
+      </c>
+      <c r="D91">
+        <v>3885</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4">
+      <c r="A92">
+        <v>2025</v>
+      </c>
+      <c r="B92" t="s">
+        <v>75</v>
+      </c>
+      <c r="C92" t="s">
+        <v>71</v>
+      </c>
+      <c r="D92">
+        <v>2228</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4">
+      <c r="A93">
+        <v>2025</v>
+      </c>
+      <c r="B93" t="s">
+        <v>75</v>
+      </c>
+      <c r="C93" t="s">
+        <v>72</v>
+      </c>
+      <c r="D93">
+        <v>1137</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4">
+      <c r="A94">
+        <v>2025</v>
+      </c>
+      <c r="B94" t="s">
+        <v>75</v>
+      </c>
+      <c r="C94" t="s">
+        <v>73</v>
+      </c>
+      <c r="D94">
+        <v>35</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC53E29E-3BCB-4B4F-89C6-6BE945E71D8E}">
   <sheetPr codeName="Hoja1"/>
   <dimension ref="A1:F160"/>
@@ -5020,7 +6413,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AC3F0BE7-B1BF-401F-81EA-ACF363BF306E}">
   <dimension ref="A1:B73"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15"/>

</xml_diff>